<commit_message>
fix: The website can only keep 4 appointment. So mofified the bulk test.
</commit_message>
<xml_diff>
--- a/data/cura_bulk_appointments.xlsx
+++ b/data/cura_bulk_appointments.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t xml:space="preserve">facility</t>
   </si>
@@ -46,7 +46,7 @@
     <t xml:space="preserve">Medicare</t>
   </si>
   <si>
-    <t xml:space="preserve">05/09/2026</t>
+    <t xml:space="preserve">05/09/2040</t>
   </si>
   <si>
     <t xml:space="preserve">Annual health check-up.</t>
@@ -61,7 +61,7 @@
     <t xml:space="preserve">Medicaid</t>
   </si>
   <si>
-    <t xml:space="preserve">08/09/2026</t>
+    <t xml:space="preserve">08/09/2040</t>
   </si>
   <si>
     <t xml:space="preserve">Routine consultation.</t>
@@ -73,52 +73,16 @@
     <t xml:space="preserve">None</t>
   </si>
   <si>
-    <t xml:space="preserve">12/09/2026</t>
+    <t xml:space="preserve">12/09/2040</t>
   </si>
   <si>
     <t xml:space="preserve">Follow-up appointment.</t>
   </si>
   <si>
-    <t xml:space="preserve">15/09/2026</t>
+    <t xml:space="preserve">15/09/2040</t>
   </si>
   <si>
     <t xml:space="preserve">General medical examination.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19/09/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Post-treatment control.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22/09/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blood pressure review.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26/09/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laboratory result discussion.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29/09/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preventive care visit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">03/10/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medication review.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07/10/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Final follow-up visit.</t>
   </si>
 </sst>
 </file>
@@ -135,6 +99,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -187,7 +152,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -252,17 +217,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFD9E7E7"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB7CCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -293,52 +247,48 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -401,7 +351,7 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF117A79"/>
-      <rgbColor rgb="FFB7CCCC"/>
+      <rgbColor rgb="FFC0C0C0"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
@@ -449,7 +399,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AppointmentsTable" displayName="AppointmentsTable" ref="A1:E11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AppointmentsTable" displayName="AppointmentsTable" ref="A1:E5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="5">
     <tableColumn id="1" name="facility"/>
     <tableColumn id="2" name="hospitalReadmission"/>
@@ -634,214 +584,118 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E1048576"/>
   <sheetFormatPr defaultColWidth="9.60546875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="27.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="38.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="38.6"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="22" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="22" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="8" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="22" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="8" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="22" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="22" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="22" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="22" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="22" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="22" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A2:A100" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A2:A94" type="list">
       <formula1>"Tokyo CURA Healthcare Center,Hongkong CURA Healthcare Center,Seoul CURA Healthcare Center"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B2:B100" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B2:B94" type="list">
       <formula1>"true,false"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C2:C100" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C2:C94" type="list">
       <formula1>"Medicare,Medicaid,None"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>